<commit_message>
Charge neighbour discovery (one HELLO per node) and the average-energy beacon of v8; re-run every result and rebuild all documents
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019rZdtfEbJpAbmcB9G79J6K
</commit_message>
<xml_diff>
--- a/thesis-final/Literature_Review_Comparison.xlsx
+++ b/thesis-final/Literature_Review_Comparison.xlsx
@@ -3624,7 +3624,7 @@
       </c>
       <c r="Q5" s="20" t="n">
         <f aca="false">$N$14/N5-1</f>
-        <v>0.808387563268257</v>
+        <v>0.768618944323934</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3670,17 +3670,17 @@
         <v>278</v>
       </c>
       <c r="N6" s="21" t="n">
-        <v>634</v>
+        <v>658</v>
       </c>
       <c r="O6" s="21" t="n">
-        <v>1883</v>
+        <v>1875</v>
       </c>
       <c r="P6" s="23" t="n">
-        <v>0.996845</v>
+        <v>0.996512</v>
       </c>
       <c r="Q6" s="25" t="n">
         <f aca="false">$N$14/N6-1</f>
-        <v>2.94479495268139</v>
+        <v>2.71732522796353</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3736,7 +3736,7 @@
       </c>
       <c r="Q7" s="20" t="n">
         <f aca="false">$N$14/N7-1</f>
-        <v>0.888972809667674</v>
+        <v>0.847432024169184</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3792,7 +3792,7 @@
       </c>
       <c r="Q8" s="25" t="n">
         <f aca="false">$N$14/N8-1</f>
-        <v>0.689864864864865</v>
+        <v>0.652702702702703</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3848,7 +3848,7 @@
       </c>
       <c r="Q9" s="20" t="n">
         <f aca="false">$N$14/N9-1</f>
-        <v>0.697895451459606</v>
+        <v>0.660556687033266</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3894,17 +3894,17 @@
         <v>285</v>
       </c>
       <c r="N10" s="21" t="n">
-        <v>1368</v>
+        <v>1335</v>
       </c>
       <c r="O10" s="21" t="n">
-        <v>1767</v>
+        <v>1766</v>
       </c>
       <c r="P10" s="23" t="n">
-        <v>0.995064</v>
+        <v>0.996207</v>
       </c>
       <c r="Q10" s="25" t="n">
         <f aca="false">$N$14/N10-1</f>
-        <v>0.828216374269006</v>
+        <v>0.832209737827715</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4025,13 +4025,13 @@
         <v>291</v>
       </c>
       <c r="N14" s="26" t="n">
-        <v>2501</v>
+        <v>2446</v>
       </c>
       <c r="O14" s="26" t="n">
-        <v>2631</v>
+        <v>2566</v>
       </c>
       <c r="P14" s="27" t="n">
-        <v>0.996392</v>
+        <v>0.997168</v>
       </c>
       <c r="Q14" s="11" t="s">
         <v>136</v>

</xml_diff>